<commit_message>
Updating the Test Plan, setuping the Test Case folders
</commit_message>
<xml_diff>
--- a/E-Commerce Web/Amazon/Test Suites/Test Case Template.xlsx
+++ b/E-Commerce Web/Amazon/Test Suites/Test Case Template.xlsx
@@ -19,20 +19,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Preconditions</t>
   </si>
   <si>
-    <t>Description</t>
-  </si>
-  <si>
     <t>Test Case Steps</t>
   </si>
   <si>
@@ -42,9 +33,6 @@
     <t>Status</t>
   </si>
   <si>
-    <t>Commentary</t>
-  </si>
-  <si>
     <t>1.</t>
   </si>
   <si>
@@ -52,6 +40,21 @@
   </si>
   <si>
     <t>3.</t>
+  </si>
+  <si>
+    <t>Test Case ID</t>
+  </si>
+  <si>
+    <t>Test Case Title</t>
+  </si>
+  <si>
+    <t>Test Case Description</t>
+  </si>
+  <si>
+    <t>Comments</t>
+  </si>
+  <si>
+    <t>Test Case Type</t>
   </si>
 </sst>
 </file>
@@ -75,7 +78,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -144,16 +147,28 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -161,6 +176,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -443,233 +461,272 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A3:I20"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.44140625" customWidth="1"/>
-    <col min="2" max="2" width="3.6640625" customWidth="1"/>
-    <col min="3" max="3" width="6.44140625" customWidth="1"/>
-    <col min="4" max="4" width="12.109375" customWidth="1"/>
-    <col min="5" max="5" width="11.5546875" customWidth="1"/>
-    <col min="6" max="6" width="14.109375" customWidth="1"/>
+    <col min="2" max="2" width="11.88671875" customWidth="1"/>
+    <col min="3" max="3" width="13.21875" customWidth="1"/>
+    <col min="4" max="4" width="13.88671875" customWidth="1"/>
+    <col min="5" max="5" width="21.109375" customWidth="1"/>
+    <col min="6" max="6" width="21.77734375" customWidth="1"/>
     <col min="7" max="7" width="13.88671875" customWidth="1"/>
-    <col min="8" max="8" width="7.109375" customWidth="1"/>
-    <col min="9" max="9" width="12.109375" customWidth="1"/>
+    <col min="8" max="8" width="16.21875" customWidth="1"/>
+    <col min="9" max="9" width="10.33203125" customWidth="1"/>
+    <col min="10" max="10" width="10.88671875" customWidth="1"/>
+    <col min="12" max="12" width="10.77734375" customWidth="1"/>
+    <col min="13" max="13" width="13.77734375" customWidth="1"/>
+    <col min="14" max="14" width="8.77734375" customWidth="1"/>
+    <col min="15" max="15" width="16.5546875" customWidth="1"/>
+    <col min="16" max="16" width="9.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B3" s="1" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="4"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="5"/>
+      <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="F2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="J2" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="5"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="5"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="5"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="2"/>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="10"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="6"/>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
       <c r="E6" s="7"/>
-      <c r="F6" s="4" t="s">
-        <v>10</v>
-      </c>
+      <c r="F6" s="7"/>
       <c r="G6" s="7"/>
       <c r="H6" s="7"/>
       <c r="I6" s="7"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
+      <c r="J6" s="7"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="I4:I6"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="C4:C6"/>
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="E4:E6"/>
-    <mergeCell ref="G4:G6"/>
-    <mergeCell ref="H4:H6"/>
+  <mergeCells count="8">
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="C3:C5"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="H3:H5"/>
+    <mergeCell ref="I3:I5"/>
+    <mergeCell ref="F3:F5"/>
+    <mergeCell ref="J3:J5"/>
+    <mergeCell ref="D3:D5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>